<commit_message>
Power Query Intro in Excel
</commit_message>
<xml_diff>
--- a/Excel/6_Advanced_Analysis/1_Analysis_Add-ins.xlsx
+++ b/Excel/6_Advanced_Analysis/1_Analysis_Add-ins.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80BB7301-AA56-41B0-AF0F-0F94E7EB3A97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4D7BF251-5D60-49D3-B801-789BF419F8C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{6C37AC85-509F-4D10-9DB1-F70D16D6FBAB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{6C37AC85-509F-4D10-9DB1-F70D16D6FBAB}"/>
   </bookViews>
   <sheets>
     <sheet name="Forecast_Original" sheetId="7" r:id="rId1"/>
@@ -64,6 +64,7 @@
     <definedName name="Year4">'What-If_Analysis'!$C$13</definedName>
   </definedNames>
   <calcPr calcId="191029" calcMode="manual"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -947,21 +948,21 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="10" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -15870,10 +15871,10 @@
   <sheetData>
     <row r="1" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B2" s="56" t="s">
+      <c r="B2" s="63" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="57"/>
+      <c r="C2" s="64"/>
       <c r="E2" s="40" t="s">
         <v>30</v>
       </c>
@@ -15963,10 +15964,10 @@
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B7" s="56" t="s">
+      <c r="B7" s="63" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="57"/>
+      <c r="C7" s="64"/>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
@@ -16377,30 +16378,30 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="59" t="s">
+      <c r="B15" s="57" t="s">
         <v>47</v>
       </c>
-      <c r="C15" s="59" t="s">
+      <c r="C15" s="57" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="59" t="s">
+      <c r="D15" s="57" t="s">
         <v>49</v>
       </c>
-      <c r="E15" s="59" t="s">
+      <c r="E15" s="57" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="58" t="s">
+      <c r="B16" s="56" t="s">
         <v>29</v>
       </c>
-      <c r="C16" s="58" t="s">
+      <c r="C16" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="D16" s="61">
+      <c r="D16" s="59">
         <v>622877.09440000006</v>
       </c>
-      <c r="E16" s="61">
+      <c r="E16" s="59">
         <v>640000.14523942047</v>
       </c>
     </row>
@@ -16410,53 +16411,53 @@
       </c>
     </row>
     <row r="20" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="59" t="s">
+      <c r="B20" s="57" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="59" t="s">
+      <c r="C20" s="57" t="s">
         <v>48</v>
       </c>
-      <c r="D20" s="59" t="s">
+      <c r="D20" s="57" t="s">
         <v>49</v>
       </c>
-      <c r="E20" s="59" t="s">
+      <c r="E20" s="57" t="s">
         <v>50</v>
       </c>
-      <c r="F20" s="59" t="s">
+      <c r="F20" s="57" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B21" s="60" t="s">
+      <c r="B21" s="58" t="s">
         <v>57</v>
       </c>
-      <c r="C21" s="60" t="s">
+      <c r="C21" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="D21" s="62">
+      <c r="D21" s="60">
         <v>0.15</v>
       </c>
-      <c r="E21" s="62">
+      <c r="E21" s="60">
         <v>0.17283479610661426</v>
       </c>
-      <c r="F21" s="60" t="s">
+      <c r="F21" s="58" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="58" t="s">
+      <c r="B22" s="56" t="s">
         <v>59</v>
       </c>
-      <c r="C22" s="58" t="s">
+      <c r="C22" s="56" t="s">
         <v>16</v>
       </c>
-      <c r="D22" s="63">
+      <c r="D22" s="61">
         <v>0.04</v>
       </c>
-      <c r="E22" s="63">
+      <c r="E22" s="61">
         <v>4.3731865887940702E-2</v>
       </c>
-      <c r="F22" s="58" t="s">
+      <c r="F22" s="56" t="s">
         <v>58</v>
       </c>
     </row>
@@ -16466,82 +16467,82 @@
       </c>
     </row>
     <row r="26" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="59" t="s">
+      <c r="B26" s="57" t="s">
         <v>47</v>
       </c>
-      <c r="C26" s="59" t="s">
+      <c r="C26" s="57" t="s">
         <v>48</v>
       </c>
-      <c r="D26" s="59" t="s">
+      <c r="D26" s="57" t="s">
         <v>54</v>
       </c>
-      <c r="E26" s="59" t="s">
+      <c r="E26" s="57" t="s">
         <v>55</v>
       </c>
-      <c r="F26" s="59" t="s">
+      <c r="F26" s="57" t="s">
         <v>56</v>
       </c>
-      <c r="G26" s="59" t="s">
+      <c r="G26" s="57" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B27" s="60" t="s">
+      <c r="B27" s="58" t="s">
         <v>29</v>
       </c>
-      <c r="C27" s="60" t="s">
+      <c r="C27" s="58" t="s">
         <v>35</v>
       </c>
-      <c r="D27" s="64">
+      <c r="D27" s="62">
         <v>640000.14523942047</v>
       </c>
-      <c r="E27" s="60" t="s">
+      <c r="E27" s="58" t="s">
         <v>60</v>
       </c>
-      <c r="F27" s="60" t="s">
+      <c r="F27" s="58" t="s">
         <v>61</v>
       </c>
-      <c r="G27" s="60">
+      <c r="G27" s="58">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B28" s="60" t="s">
+      <c r="B28" s="58" t="s">
         <v>57</v>
       </c>
-      <c r="C28" s="60" t="s">
+      <c r="C28" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="D28" s="62">
+      <c r="D28" s="60">
         <v>0.17283479610661426</v>
       </c>
-      <c r="E28" s="60" t="s">
+      <c r="E28" s="58" t="s">
         <v>67</v>
       </c>
-      <c r="F28" s="60" t="s">
+      <c r="F28" s="58" t="s">
         <v>62</v>
       </c>
-      <c r="G28" s="60">
+      <c r="G28" s="58">
         <v>2.7165203893385753E-2</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="58" t="s">
+      <c r="B29" s="56" t="s">
         <v>59</v>
       </c>
-      <c r="C29" s="58" t="s">
+      <c r="C29" s="56" t="s">
         <v>16</v>
       </c>
-      <c r="D29" s="63">
+      <c r="D29" s="61">
         <v>4.3731865887940702E-2</v>
       </c>
-      <c r="E29" s="58" t="s">
+      <c r="E29" s="56" t="s">
         <v>68</v>
       </c>
-      <c r="F29" s="58" t="s">
+      <c r="F29" s="56" t="s">
         <v>62</v>
       </c>
-      <c r="G29" s="58">
+      <c r="G29" s="56">
         <v>6.2681341120593009E-3</v>
       </c>
     </row>

</xml_diff>